<commit_message>
Update Nội dung công việc hàng ngày.xlsx
</commit_message>
<xml_diff>
--- a/5. Other/Nội dung công việc hàng ngày.xlsx
+++ b/5. Other/Nội dung công việc hàng ngày.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VNET\5. Other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5389BC2F-1CA5-4E4D-94A6-D04BE5237CD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{100DCEA3-4DBD-41BB-B98D-35031B4CDE34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{F20CEA29-D7AE-4CD4-9104-84E191A61AC3}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="32">
   <si>
     <t>Hoàn thiện 73 dây nguồn VNSH03</t>
   </si>
@@ -107,6 +107,24 @@
   </si>
   <si>
     <t>Nhận 9 LE nâng cấp 2G-&gt;4G anh Tuấn BG</t>
+  </si>
+  <si>
+    <t>Nhập kho 23 thiết bị VNSH03</t>
+  </si>
+  <si>
+    <t>Nhập kho 100 RFID</t>
+  </si>
+  <si>
+    <t>Xuất 100 anten GSM + GPS + dây nguồn LE trong tổng là 300/500</t>
+  </si>
+  <si>
+    <t>Nhận 1 ACT-01 từ kho dán lại tem đã trả trong ngày</t>
+  </si>
+  <si>
+    <t>Xuất kho 80 nắp chặn quạt gió, 10 nắp chặn nguồn vỏ hộp VNSH03 gửi qua X-Force (A. Cảnh)</t>
+  </si>
+  <si>
+    <t>Xuất linh kiện BH chưa trả kho phiếu (thứ 06/06/26 làm phiếu trả sau)</t>
   </si>
 </sst>
 </file>
@@ -259,7 +277,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -268,6 +286,36 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -285,25 +333,22 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="17" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -315,25 +360,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -658,15 +691,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="10">
+      <c r="A1" s="8">
         <v>46174</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -675,146 +708,146 @@
       <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="14"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="12"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="9">
+      <c r="A3" s="6">
         <v>46202</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="9"/>
-      <c r="B4" s="15"/>
-      <c r="C4" s="15" t="s">
+      <c r="A4" s="6"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="9"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15" t="s">
+      <c r="A5" s="6"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="9"/>
-      <c r="B6" s="15" t="s">
+      <c r="A6" s="6"/>
+      <c r="B6" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="9"/>
-      <c r="B7" s="15"/>
-      <c r="C7" s="15" t="s">
+      <c r="A7" s="6"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="15"/>
-      <c r="E7" s="15"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="9"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15" t="s">
+      <c r="A8" s="6"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="9">
+      <c r="A9" s="6">
         <v>46203</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="5"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="15"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="9"/>
-      <c r="B10" s="15"/>
-      <c r="C10" s="6" t="s">
+      <c r="A10" s="6"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="8"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="18"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="9"/>
-      <c r="B11" s="15"/>
-      <c r="C11" s="6" t="s">
+      <c r="A11" s="6"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="8"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="18"/>
     </row>
     <row r="12" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="9"/>
-      <c r="B12" s="15"/>
-      <c r="C12" s="6" t="s">
+      <c r="A12" s="6"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="8"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="18"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="9"/>
+      <c r="A13" s="6"/>
       <c r="B13" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="8"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="18"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:G8" xr:uid="{5B424F82-FB95-405B-80D1-35D47957B3B0}">
@@ -824,6 +857,8 @@
     <filterColumn colId="5" showButton="0"/>
   </autoFilter>
   <mergeCells count="18">
+    <mergeCell ref="C12:G12"/>
+    <mergeCell ref="C13:G13"/>
     <mergeCell ref="A9:A13"/>
     <mergeCell ref="B9:B12"/>
     <mergeCell ref="A3:A8"/>
@@ -840,8 +875,6 @@
     <mergeCell ref="C9:G9"/>
     <mergeCell ref="C10:G10"/>
     <mergeCell ref="C11:G11"/>
-    <mergeCell ref="C12:G12"/>
-    <mergeCell ref="C13:G13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -849,25 +882,25 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50B04270-3E3B-4748-8F06-1DEA88575B23}">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="36.7109375" customWidth="1"/>
+    <col min="3" max="3" width="45.28515625" customWidth="1"/>
     <col min="7" max="7" width="9.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="16">
+      <c r="A1" s="25">
         <v>46204</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -876,149 +909,237 @@
       <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="9">
+      <c r="A3" s="6">
         <v>46204</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
     </row>
     <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="9"/>
-      <c r="B4" s="15" t="s">
+      <c r="A4" s="6"/>
+      <c r="B4" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="9"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15" t="s">
+      <c r="A5" s="6"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="9"/>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15" t="s">
+      <c r="A6" s="6"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="20">
+      <c r="A7" s="19">
         <v>46205</v>
       </c>
-      <c r="B7" s="23" t="s">
+      <c r="B7" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="5"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="15"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="21"/>
-      <c r="B8" s="24"/>
-      <c r="C8" s="6" t="s">
+      <c r="A8" s="20"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="8"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="18"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="21"/>
-      <c r="B9" s="25"/>
-      <c r="C9" s="6" t="s">
+      <c r="A9" s="20"/>
+      <c r="B9" s="24"/>
+      <c r="C9" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="8"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="18"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="21"/>
-      <c r="B10" s="19" t="s">
+      <c r="A10" s="20"/>
+      <c r="B10" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="8"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="18"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="21"/>
-      <c r="B11" s="19"/>
-      <c r="C11" s="6" t="s">
+      <c r="A11" s="20"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="8"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="18"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="21"/>
-      <c r="B12" s="19"/>
-      <c r="C12" s="6" t="s">
+      <c r="A12" s="20"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="8"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="18"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="22"/>
-      <c r="B13" s="19"/>
-      <c r="C13" s="6" t="s">
+      <c r="A13" s="21"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="8"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="18"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="28">
+        <v>46206</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="5"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="29"/>
+      <c r="B15" s="23"/>
+      <c r="C15" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="15"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="29"/>
+      <c r="B16" s="23"/>
+      <c r="C16" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="15"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="29"/>
+      <c r="B17" s="24"/>
+      <c r="C17" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="14"/>
+      <c r="G17" s="15"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="29"/>
+      <c r="B18" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="15"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="30"/>
+      <c r="B19" s="24"/>
+      <c r="C19" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="15"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="26">
+    <mergeCell ref="C15:G15"/>
+    <mergeCell ref="C17:G17"/>
+    <mergeCell ref="C19:G19"/>
+    <mergeCell ref="C16:G16"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C18:G18"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="A14:A19"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="A3:A6"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="C5:G5"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="C6:G6"/>
     <mergeCell ref="C7:G7"/>
     <mergeCell ref="A7:A13"/>
     <mergeCell ref="B7:B9"/>
@@ -1029,14 +1150,6 @@
     <mergeCell ref="C11:G11"/>
     <mergeCell ref="C12:G12"/>
     <mergeCell ref="C13:G13"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="C2:G2"/>
-    <mergeCell ref="A3:A6"/>
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="C5:G5"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="C6:G6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>